<commit_message>
Trying out some petal sprites
</commit_message>
<xml_diff>
--- a/.Notes/leves.xlsx
+++ b/.Notes/leves.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programs\Steam\Steam\steamapps\common\Stardew Valley\SiMods\[Si]\CBLeaves\.Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C267F300-3588-443A-86A4-C2859741A1AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC41C658-5BE8-4A32-8347-CE05E689E440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Leaves" sheetId="1" r:id="rId1"/>
+    <sheet name="Flowers" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="126">
   <si>
     <t>Leaf</t>
   </si>
@@ -303,6 +304,117 @@
   </si>
   <si>
     <t>Sea buckthorn bush</t>
+  </si>
+  <si>
+    <t>Crocus</t>
+  </si>
+  <si>
+    <t>Dandelion</t>
+  </si>
+  <si>
+    <t>Daffodil</t>
+  </si>
+  <si>
+    <t>Sweet Pea</t>
+  </si>
+  <si>
+    <t>Cherry Blossom</t>
+  </si>
+  <si>
+    <t>Cactus Flower</t>
+  </si>
+  <si>
+    <t>Tulip</t>
+  </si>
+  <si>
+    <t>Blue Jazz</t>
+  </si>
+  <si>
+    <t>Spangle</t>
+  </si>
+  <si>
+    <t>Poppy</t>
+  </si>
+  <si>
+    <t>Fairy Rose</t>
+  </si>
+  <si>
+    <t>Sunflower</t>
+  </si>
+  <si>
+    <t>Prize is flowers on head hat</t>
+  </si>
+  <si>
+    <t>red</t>
+  </si>
+  <si>
+    <t>yellow</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>dark blue</t>
+  </si>
+  <si>
+    <t>light blue</t>
+  </si>
+  <si>
+    <t>pink</t>
+  </si>
+  <si>
+    <t>violet</t>
+  </si>
+  <si>
+    <t>teal</t>
+  </si>
+  <si>
+    <t>periwinkle</t>
+  </si>
+  <si>
+    <t>indigo</t>
+  </si>
+  <si>
+    <t>pastel</t>
+  </si>
+  <si>
+    <t>sky blue</t>
+  </si>
+  <si>
+    <t>Common</t>
+  </si>
+  <si>
+    <t>Uncommon</t>
+  </si>
+  <si>
+    <t>Very rare</t>
+  </si>
+  <si>
+    <t>Rare</t>
+  </si>
+  <si>
+    <t>Uncommmon</t>
+  </si>
+  <si>
+    <t>Exquisite</t>
+  </si>
+  <si>
+    <t>Very Rare</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Desert Rose</t>
+  </si>
+  <si>
+    <t>Book in trees at high altitudes</t>
+  </si>
+  <si>
+    <t>Book on magical tree properties</t>
+  </si>
+  <si>
+    <t>Book on trees around the world/greenhousing trees</t>
   </si>
 </sst>
 </file>
@@ -649,6 +761,9 @@
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="16.109375" customWidth="1"/>
     <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="9" max="9" width="11.21875" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -752,6 +867,12 @@
       <c r="B12" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="D12" s="1">
+        <v>27</v>
+      </c>
+      <c r="E12" s="3">
+        <v>24</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
@@ -1077,6 +1198,15 @@
       <c r="D30" t="s">
         <v>56</v>
       </c>
+      <c r="F30" t="s">
+        <v>123</v>
+      </c>
+      <c r="I30" t="s">
+        <v>124</v>
+      </c>
+      <c r="L30" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
@@ -1231,6 +1361,315 @@
       </c>
       <c r="D52" t="s">
         <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E42EC66B-C337-40A3-BF49-C636A0690182}">
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F9" t="s">
+        <v>117</v>
+      </c>
+      <c r="G9" t="s">
+        <v>120</v>
+      </c>
+      <c r="H9" t="s">
+        <v>114</v>
+      </c>
+      <c r="I9" t="s">
+        <v>117</v>
+      </c>
+      <c r="J9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="L10" t="s">
+        <v>116</v>
+      </c>
+      <c r="M10" t="s">
+        <v>93</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>103</v>
+      </c>
+      <c r="F11" t="s">
+        <v>102</v>
+      </c>
+      <c r="G11" t="s">
+        <v>107</v>
+      </c>
+      <c r="H11" t="s">
+        <v>112</v>
+      </c>
+      <c r="I11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L11" t="s">
+        <v>114</v>
+      </c>
+      <c r="M11" t="s">
+        <v>90</v>
+      </c>
+      <c r="N11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>96</v>
+      </c>
+      <c r="D12">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>111</v>
+      </c>
+      <c r="F12" t="s">
+        <v>105</v>
+      </c>
+      <c r="G12" t="s">
+        <v>104</v>
+      </c>
+      <c r="H12" t="s">
+        <v>106</v>
+      </c>
+      <c r="I12" t="s">
+        <v>113</v>
+      </c>
+      <c r="J12" t="s">
+        <v>108</v>
+      </c>
+      <c r="L12" t="s">
+        <v>114</v>
+      </c>
+      <c r="M12" t="s">
+        <v>91</v>
+      </c>
+      <c r="N12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>97</v>
+      </c>
+      <c r="D13">
+        <v>6</v>
+      </c>
+      <c r="E13" t="s">
+        <v>103</v>
+      </c>
+      <c r="F13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G13" t="s">
+        <v>107</v>
+      </c>
+      <c r="H13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I13" t="s">
+        <v>109</v>
+      </c>
+      <c r="J13" t="s">
+        <v>108</v>
+      </c>
+      <c r="L13" t="s">
+        <v>114</v>
+      </c>
+      <c r="M13" t="s">
+        <v>92</v>
+      </c>
+      <c r="N13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>98</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>103</v>
+      </c>
+      <c r="F14" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" t="s">
+        <v>104</v>
+      </c>
+      <c r="L14" t="s">
+        <v>114</v>
+      </c>
+      <c r="M14" t="s">
+        <v>89</v>
+      </c>
+      <c r="N14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>111</v>
+      </c>
+      <c r="F15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" t="s">
+        <v>107</v>
+      </c>
+      <c r="H15" t="s">
+        <v>106</v>
+      </c>
+      <c r="I15" t="s">
+        <v>110</v>
+      </c>
+      <c r="J15" t="s">
+        <v>108</v>
+      </c>
+      <c r="L15" t="s">
+        <v>115</v>
+      </c>
+      <c r="M15" t="s">
+        <v>94</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>103</v>
+      </c>
+      <c r="N16">
+        <f>SUM(N10:N15)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D17">
+        <f>SUM(D11:D16)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="H19" t="s">
+        <v>121</v>
+      </c>
+      <c r="I19">
+        <f>SUM(D17+N16)</f>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made flower and plum leaf sprites
</commit_message>
<xml_diff>
--- a/.Notes/leves.xlsx
+++ b/.Notes/leves.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programs\Steam\Steam\steamapps\common\Stardew Valley\SiMods\[Si]\CBLeaves\.Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C08572C-EB3C-4923-892E-D03DA0943840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CBCAF04-3A33-4218-A91E-1CA4E8549CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="140">
   <si>
     <t>Leaf</t>
   </si>
@@ -448,6 +448,15 @@
   </si>
   <si>
     <t>Rain</t>
+  </si>
+  <si>
+    <t>Plum</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Summer/Fall</t>
   </si>
 </sst>
 </file>
@@ -788,7 +797,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -799,7 +808,7 @@
     <col min="12" max="12" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -810,7 +819,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -820,24 +829,42 @@
       <c r="F2" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N2" t="s">
+        <v>91</v>
+      </c>
+      <c r="O2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N3" t="s">
+        <v>90</v>
+      </c>
+      <c r="O3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="F4" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N4" t="s">
+        <v>92</v>
+      </c>
+      <c r="O4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -847,24 +874,42 @@
       <c r="F5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N5" t="s">
+        <v>89</v>
+      </c>
+      <c r="O5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F6" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N6" t="s">
+        <v>137</v>
+      </c>
+      <c r="O6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="F7" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N7" t="s">
+        <v>96</v>
+      </c>
+      <c r="O7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -874,29 +919,53 @@
       <c r="F8" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N8" t="s">
+        <v>95</v>
+      </c>
+      <c r="O8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F9" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N9" t="s">
+        <v>97</v>
+      </c>
+      <c r="O9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N10" t="s">
+        <v>98</v>
+      </c>
+      <c r="O10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N11" t="s">
+        <v>100</v>
+      </c>
+      <c r="O11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>5</v>
       </c>
@@ -906,13 +975,19 @@
       <c r="E12" s="3">
         <v>26</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="N12" t="s">
+        <v>99</v>
+      </c>
+      <c r="O12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -923,7 +998,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
@@ -931,7 +1006,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Added rewards file and flower plus more forage leaves
</commit_message>
<xml_diff>
--- a/.Notes/leves.xlsx
+++ b/.Notes/leves.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programs\Steam\Steam\steamapps\common\Stardew Valley\SiMods\[Si]\CBLeaves\.Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CBCAF04-3A33-4218-A91E-1CA4E8549CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0616849C-364D-448F-8390-43ECC79CAC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="144">
   <si>
     <t>Leaf</t>
   </si>
@@ -457,6 +457,18 @@
   </si>
   <si>
     <t>Summer/Fall</t>
+  </si>
+  <si>
+    <t>luau skirt</t>
+  </si>
+  <si>
+    <t>grass skirt</t>
+  </si>
+  <si>
+    <t>living hat</t>
+  </si>
+  <si>
+    <t>all</t>
   </si>
 </sst>
 </file>
@@ -797,7 +809,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -958,6 +970,15 @@
       <c r="B11" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="D11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E11" t="s">
+        <v>141</v>
+      </c>
+      <c r="F11" t="s">
+        <v>142</v>
+      </c>
       <c r="N11" t="s">
         <v>100</v>
       </c>
@@ -970,10 +991,13 @@
         <v>5</v>
       </c>
       <c r="D12" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E12" s="3">
-        <v>26</v>
+        <v>29</v>
+      </c>
+      <c r="F12" t="s">
+        <v>143</v>
       </c>
       <c r="N12" t="s">
         <v>99</v>
@@ -1369,7 +1393,7 @@
       <c r="A33" t="s">
         <v>16</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1521,6 +1545,70 @@
       </c>
       <c r="B54" s="3" t="s">
         <v>136</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>90</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>95</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>97</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>98</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>100</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>99</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>137</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made grass hat and a bunch of SVE leaf sprites
</commit_message>
<xml_diff>
--- a/.Notes/leves.xlsx
+++ b/.Notes/leves.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programs\Steam\Steam\steamapps\common\Stardew Valley\SiMods\[Si]\CBLeaves\.Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0616849C-364D-448F-8390-43ECC79CAC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514C47B7-6211-47CA-ADE2-2A718D4776B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="163">
   <si>
     <t>Leaf</t>
   </si>
@@ -243,9 +243,6 @@
     <t>Nectarine tree</t>
   </si>
   <si>
-    <t>Money tree?</t>
-  </si>
-  <si>
     <t>RSV</t>
   </si>
   <si>
@@ -420,12 +417,6 @@
     <t>Bearberry</t>
   </si>
   <si>
-    <t>Baneberry</t>
-  </si>
-  <si>
-    <t>Salal berry</t>
-  </si>
-  <si>
     <t>summer</t>
   </si>
   <si>
@@ -469,13 +460,79 @@
   </si>
   <si>
     <t>all</t>
+  </si>
+  <si>
+    <t>A summit forage or potions</t>
+  </si>
+  <si>
+    <t>VMV books</t>
+  </si>
+  <si>
+    <t>Essences maybe?</t>
+  </si>
+  <si>
+    <t>Money tree</t>
+  </si>
+  <si>
+    <t>paper birch</t>
+  </si>
+  <si>
+    <t>spring</t>
+  </si>
+  <si>
+    <t>Slime Berry</t>
+  </si>
+  <si>
+    <t>Thistle</t>
+  </si>
+  <si>
+    <t>Joja leaf</t>
+  </si>
+  <si>
+    <t>Monster Fruit</t>
+  </si>
+  <si>
+    <t>why does it feel like this leaf is watching you?'</t>
+  </si>
+  <si>
+    <t>this leaf is dripping with slime'</t>
+  </si>
+  <si>
+    <t>this leaf feels like plastic'</t>
+  </si>
+  <si>
+    <t>Dewdrop Berry</t>
+  </si>
+  <si>
+    <t>Goldenrod</t>
+  </si>
+  <si>
+    <t>sum/fal</t>
+  </si>
+  <si>
+    <t>Winter Star Rose</t>
+  </si>
+  <si>
+    <t>Swamp Flower</t>
+  </si>
+  <si>
+    <t>water leaf</t>
+  </si>
+  <si>
+    <t>Salal Berry</t>
+  </si>
+  <si>
+    <t>Primrose</t>
+  </si>
+  <si>
+    <t>spr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -487,6 +544,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -524,11 +587,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -842,10 +906,10 @@
         <v>46</v>
       </c>
       <c r="N2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
@@ -856,7 +920,7 @@
         <v>47</v>
       </c>
       <c r="N3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O3" t="s">
         <v>3</v>
@@ -870,10 +934,10 @@
         <v>48</v>
       </c>
       <c r="N4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -887,7 +951,7 @@
         <v>49</v>
       </c>
       <c r="N5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O5" t="s">
         <v>9</v>
@@ -901,7 +965,7 @@
         <v>52</v>
       </c>
       <c r="N6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="O6" t="s">
         <v>5</v>
@@ -915,10 +979,10 @@
         <v>53</v>
       </c>
       <c r="N7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
@@ -929,10 +993,10 @@
         <v>3</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="N8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O8" t="s">
         <v>3</v>
@@ -946,7 +1010,7 @@
         <v>54</v>
       </c>
       <c r="N9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O9" t="s">
         <v>4</v>
@@ -957,7 +1021,7 @@
         <v>5</v>
       </c>
       <c r="N10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O10" t="s">
         <v>4</v>
@@ -971,19 +1035,19 @@
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O11" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
@@ -997,10 +1061,10 @@
         <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="N12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O12" t="s">
         <v>5</v>
@@ -1059,10 +1123,10 @@
         <v>63</v>
       </c>
       <c r="J17">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="L17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M17">
         <v>23</v>
@@ -1079,16 +1143,16 @@
         <v>59</v>
       </c>
       <c r="G18" t="s">
-        <v>70</v>
-      </c>
-      <c r="I18" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>64</v>
       </c>
       <c r="J18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="M18">
         <v>3</v>
@@ -1105,16 +1169,16 @@
         <v>60</v>
       </c>
       <c r="G19" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="J19" t="s">
         <v>70</v>
       </c>
-      <c r="I19" t="s">
-        <v>65</v>
-      </c>
-      <c r="J19" t="s">
-        <v>71</v>
-      </c>
       <c r="L19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M19">
         <v>3</v>
@@ -1131,16 +1195,16 @@
         <v>61</v>
       </c>
       <c r="G20" t="s">
-        <v>71</v>
-      </c>
-      <c r="I20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I20" s="3" t="s">
         <v>66</v>
       </c>
       <c r="J20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M20">
         <v>3</v>
@@ -1160,16 +1224,16 @@
         <v>62</v>
       </c>
       <c r="G21" t="s">
-        <v>71</v>
-      </c>
-      <c r="I21" t="s">
+        <v>70</v>
+      </c>
+      <c r="I21" s="3" t="s">
         <v>67</v>
       </c>
       <c r="J21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="M21">
         <v>2</v>
@@ -1183,19 +1247,19 @@
         <v>4</v>
       </c>
       <c r="F22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G22" t="s">
-        <v>74</v>
-      </c>
-      <c r="I22" t="s">
-        <v>68</v>
+        <v>73</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>144</v>
       </c>
       <c r="J22" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M22">
         <v>3</v>
@@ -1209,19 +1273,22 @@
         <v>5</v>
       </c>
       <c r="F23" t="s">
+        <v>72</v>
+      </c>
+      <c r="G23" t="s">
         <v>73</v>
       </c>
-      <c r="G23" t="s">
-        <v>74</v>
-      </c>
-      <c r="I23" t="s">
+      <c r="H23" t="s">
+        <v>145</v>
+      </c>
+      <c r="I23" s="3" t="s">
         <v>62</v>
       </c>
       <c r="J23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M23">
         <v>3</v>
@@ -1235,22 +1302,22 @@
         <v>9</v>
       </c>
       <c r="F24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G24" t="s">
-        <v>70</v>
-      </c>
-      <c r="I24" t="s">
-        <v>126</v>
+        <v>69</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>125</v>
       </c>
       <c r="J24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K24" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="L24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M24">
         <v>3</v>
@@ -1267,22 +1334,25 @@
         <v>56</v>
       </c>
       <c r="F25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G25" t="s">
-        <v>74</v>
-      </c>
-      <c r="I25" t="s">
-        <v>127</v>
+        <v>73</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>147</v>
       </c>
       <c r="J25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K25" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="L25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M25">
         <v>3</v>
@@ -1296,19 +1366,19 @@
         <v>3</v>
       </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G26" t="s">
-        <v>74</v>
-      </c>
-      <c r="I26" t="s">
-        <v>128</v>
+        <v>73</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>148</v>
       </c>
       <c r="J26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K26" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
@@ -1319,19 +1389,19 @@
         <v>4</v>
       </c>
       <c r="F27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G27" t="s">
-        <v>74</v>
-      </c>
-      <c r="I27" t="s">
-        <v>132</v>
+        <v>73</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="J27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K27" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
@@ -1342,10 +1412,22 @@
         <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G28" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="J28" t="s">
+        <v>73</v>
+      </c>
+      <c r="K28" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
@@ -1355,6 +1437,18 @@
       <c r="D29" t="s">
         <v>57</v>
       </c>
+      <c r="H29" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J29" t="s">
+        <v>73</v>
+      </c>
+      <c r="K29" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
@@ -1367,13 +1461,19 @@
         <v>56</v>
       </c>
       <c r="F30" t="s">
-        <v>123</v>
-      </c>
-      <c r="I30" t="s">
+        <v>122</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="J30" t="s">
+        <v>73</v>
+      </c>
+      <c r="K30" t="s">
+        <v>140</v>
+      </c>
+      <c r="L30" t="s">
         <v>124</v>
-      </c>
-      <c r="L30" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
@@ -1383,31 +1483,85 @@
       <c r="B31" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="F31" t="s">
+        <v>142</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="J31" t="s">
+        <v>73</v>
+      </c>
+      <c r="K31" t="s">
+        <v>156</v>
+      </c>
+      <c r="L31" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="I32" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="J32" t="s">
+        <v>73</v>
+      </c>
+      <c r="K32" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>16</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="H33" t="s">
+        <v>159</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="J33" t="s">
+        <v>73</v>
+      </c>
+      <c r="K33" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="I34" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="J34" t="s">
+        <v>73</v>
+      </c>
+      <c r="K34" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="I35" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="J35" t="s">
+        <v>73</v>
+      </c>
+      <c r="K35" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>17</v>
       </c>
@@ -1415,17 +1569,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B37" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="I37" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="I38" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>18</v>
       </c>
@@ -1433,17 +1593,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B40" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -1451,12 +1611,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -1464,17 +1624,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B45" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>20</v>
       </c>
@@ -1483,7 +1643,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>21</v>
       </c>
@@ -1533,23 +1693,23 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>3</v>
@@ -1557,7 +1717,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>3</v>
@@ -1565,7 +1725,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>4</v>
@@ -1573,7 +1733,7 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>4</v>
@@ -1581,15 +1741,15 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>5</v>
@@ -1597,7 +1757,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>5</v>
@@ -1605,13 +1765,14 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1646,82 +1807,82 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G9" t="s">
+        <v>119</v>
+      </c>
+      <c r="H9" t="s">
+        <v>113</v>
+      </c>
+      <c r="I9" t="s">
+        <v>116</v>
+      </c>
+      <c r="J9" t="s">
         <v>118</v>
-      </c>
-      <c r="F9" t="s">
-        <v>117</v>
-      </c>
-      <c r="G9" t="s">
-        <v>120</v>
-      </c>
-      <c r="H9" t="s">
-        <v>114</v>
-      </c>
-      <c r="I9" t="s">
-        <v>117</v>
-      </c>
-      <c r="J9" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="L10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="M10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N10">
         <v>1</v>
@@ -1729,31 +1890,31 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D11">
         <v>5</v>
       </c>
       <c r="E11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -1761,34 +1922,34 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D12">
         <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F12" t="s">
+        <v>104</v>
+      </c>
+      <c r="G12" t="s">
+        <v>103</v>
+      </c>
+      <c r="H12" t="s">
         <v>105</v>
       </c>
-      <c r="G12" t="s">
-        <v>104</v>
-      </c>
-      <c r="H12" t="s">
-        <v>106</v>
-      </c>
       <c r="I12" t="s">
+        <v>112</v>
+      </c>
+      <c r="J12" t="s">
+        <v>107</v>
+      </c>
+      <c r="L12" t="s">
         <v>113</v>
       </c>
-      <c r="J12" t="s">
-        <v>108</v>
-      </c>
-      <c r="L12" t="s">
-        <v>114</v>
-      </c>
       <c r="M12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N12">
         <v>1</v>
@@ -1796,34 +1957,34 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D13">
         <v>6</v>
       </c>
       <c r="E13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G13" t="s">
+        <v>106</v>
+      </c>
+      <c r="H13" t="s">
+        <v>105</v>
+      </c>
+      <c r="I13" t="s">
+        <v>108</v>
+      </c>
+      <c r="J13" t="s">
         <v>107</v>
       </c>
-      <c r="H13" t="s">
-        <v>106</v>
-      </c>
-      <c r="I13" t="s">
-        <v>109</v>
-      </c>
-      <c r="J13" t="s">
-        <v>108</v>
-      </c>
       <c r="L13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N13">
         <v>1</v>
@@ -1831,25 +1992,25 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D14">
         <v>3</v>
       </c>
       <c r="E14" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G14" t="s">
         <v>103</v>
       </c>
-      <c r="F14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G14" t="s">
-        <v>104</v>
-      </c>
       <c r="L14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N14">
         <v>1</v>
@@ -1857,34 +2018,34 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D15">
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G15" t="s">
+        <v>106</v>
+      </c>
+      <c r="H15" t="s">
+        <v>105</v>
+      </c>
+      <c r="I15" t="s">
+        <v>109</v>
+      </c>
+      <c r="J15" t="s">
         <v>107</v>
       </c>
-      <c r="H15" t="s">
-        <v>106</v>
-      </c>
-      <c r="I15" t="s">
-        <v>110</v>
-      </c>
-      <c r="J15" t="s">
-        <v>108</v>
-      </c>
       <c r="L15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N15">
         <v>1</v>
@@ -1892,13 +2053,13 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="N16">
         <f>SUM(N10:N15)</f>
@@ -1913,7 +2074,7 @@
     </row>
     <row r="19" spans="4:9" x14ac:dyDescent="0.3">
       <c r="H19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I19">
         <f>SUM(D17+N16)</f>

</xml_diff>